<commit_message>
File mapper issue fixing
</commit_message>
<xml_diff>
--- a/Documents/SUBS-LN-F1H26-Translated.xlsx
+++ b/Documents/SUBS-LN-F1H26-Translated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRM 2.0\Adobe Web Forms\F1H26\Subsidairy\SEMAG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Adobe-Form-Builder-main\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B90D94-9082-4BDF-AA27-E6E900D1F01C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040CEF6E-4F12-4893-9109-625597849A23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1710" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete Translations" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="216">
-  <si>
-    <t>Translation</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="215">
   <si>
     <t>heading</t>
   </si>
@@ -228,9 +225,6 @@
   </si>
   <si>
     <t>(Do not change this column)</t>
-  </si>
-  <si>
-    <t>Original en_GB Text</t>
   </si>
   <si>
     <t>Sample Web Forms</t>
@@ -396,9 +390,6 @@
     <t>Form Thank you Page</t>
   </si>
   <si>
-    <t>Translation [Language]</t>
-  </si>
-  <si>
     <t>A1</t>
   </si>
   <si>
@@ -445,9 +436,6 @@
   </si>
   <si>
     <t>Q4</t>
-  </si>
-  <si>
-    <t>Complete this Translation Column</t>
   </si>
   <si>
     <t>Language_Country</t>
@@ -705,6 +693,15 @@
   </si>
   <si>
     <t>Divertissement</t>
+  </si>
+  <si>
+    <t>Original Text</t>
+  </si>
+  <si>
+    <t>Project Code</t>
+  </si>
+  <si>
+    <t>F1H26</t>
   </si>
 </sst>
 </file>
@@ -755,7 +752,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -792,14 +789,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -898,56 +889,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -957,62 +929,89 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1295,949 +1294,858 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" style="20" customWidth="1"/>
-    <col min="2" max="2" width="46.33203125" style="20" customWidth="1"/>
-    <col min="3" max="3" width="44.21875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="64.33203125" style="26" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="9"/>
+    <col min="1" max="1" width="25.33203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" style="21" customWidth="1"/>
+    <col min="3" max="3" width="64.33203125" style="13" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>63</v>
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>212</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="33"/>
+      <c r="B2" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="34"/>
+      <c r="B3" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="40"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="34"/>
+      <c r="B4" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="34"/>
+      <c r="B5" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="34"/>
+      <c r="B6" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="24"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="34"/>
+      <c r="B7" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="22"/>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="34"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="11"/>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="34"/>
+      <c r="B9" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="12"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="33"/>
+      <c r="B11" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="13" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="34"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="15"/>
+    </row>
+    <row r="16" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="33"/>
+      <c r="B17" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="34"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="15"/>
+    </row>
+    <row r="28" spans="1:3" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="33"/>
+      <c r="B29" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="34"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="22"/>
+    </row>
+    <row r="35" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="33"/>
+      <c r="B36" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C39" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B41" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="34"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="11"/>
+    </row>
+    <row r="43" spans="1:3" s="6" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="C43" s="25" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="33"/>
+      <c r="B44" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="C45" s="22" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B46" s="16" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="31"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="21"/>
-    </row>
-    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="32"/>
-      <c r="B3" s="40" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="35"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
-      <c r="B4" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="36" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
-      <c r="B5" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
-      <c r="B6" s="14" t="s">
+      <c r="C46" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B47" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="C47" s="22" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B48" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B50" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="34"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="10"/>
+    </row>
+    <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="34"/>
+      <c r="B54" s="16"/>
+      <c r="C54" s="11"/>
+    </row>
+    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="34"/>
+      <c r="B55" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C55" s="12"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B56" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" s="22" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C57" s="26" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B58" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="C58" s="27" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B59" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="34"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="15"/>
+    </row>
+    <row r="61" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="34"/>
+      <c r="B61" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C61" s="28"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B63" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" s="22" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" s="22" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B65" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="22" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5" t="str">
-        <f>RIGHT(C5,2)</f>
-        <v/>
-      </c>
-      <c r="D6" s="36"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
-      <c r="B7" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="22"/>
-    </row>
-    <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="32"/>
-      <c r="B8" s="14"/>
-      <c r="C8"/>
-      <c r="D8" s="23"/>
-    </row>
-    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="32"/>
-      <c r="B9" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D9" s="24"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="21" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
-      <c r="B11" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="22" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B12" s="14" t="s">
+      <c r="B66" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66" s="22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="B67" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" s="22" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" s="22" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="B69" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C69" s="22" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B70" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C70" s="22" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B71" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="22" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B72" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C72" s="22" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B73" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="C73" s="27"/>
+    </row>
+    <row r="74" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A74" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B74" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="C74" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="B75" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C75" s="22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="B76" s="16"/>
+      <c r="C76" s="15"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C77" s="22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="B78" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C78" s="26" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B79" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="C79" s="29"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B80" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C80" s="22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="22" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="22" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="32"/>
-      <c r="B15" s="14"/>
-      <c r="C15"/>
-      <c r="D15" s="23"/>
-    </row>
-    <row r="16" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
+      <c r="B81" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="B16" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="21" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="31"/>
-      <c r="B17" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="22" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="27" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="27" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="22" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="22" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="22" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="22" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="22" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="32"/>
-      <c r="B27" s="14"/>
-      <c r="C27"/>
-      <c r="D27" s="23"/>
-    </row>
-    <row r="28" spans="1:4" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="31" t="s">
+      <c r="C81" s="29" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A82" s="36" t="s">
         <v>196</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="21" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="31"/>
-      <c r="B29" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="21" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="C30" s="5"/>
-      <c r="D30" s="22" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="22" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" s="5"/>
-      <c r="D32" s="22" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="22" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="32"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="22"/>
-    </row>
-    <row r="35" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="31" t="s">
-        <v>133</v>
-      </c>
-      <c r="B35" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35" s="6"/>
-      <c r="D35" s="21" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="31"/>
-      <c r="B36" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="21" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="22" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="C38" s="5"/>
-      <c r="D38" s="22" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="22" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="22" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="B41" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="22" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="32"/>
-      <c r="B42" s="14"/>
-      <c r="C42"/>
-      <c r="D42" s="23"/>
-    </row>
-    <row r="43" spans="1:4" s="10" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="31" t="s">
+      <c r="B82" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="C82" s="30"/>
+    </row>
+    <row r="83" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A83" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="B43" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="C43" s="6"/>
-      <c r="D43" s="37" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="31"/>
-      <c r="B44" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C44" s="6"/>
-      <c r="D44" s="21" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B45" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="22" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="B46" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C46" s="5"/>
-      <c r="D46" s="22" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="B47" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C47" s="5"/>
-      <c r="D47" s="22" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="22" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="C49"/>
-      <c r="D49" s="22" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="B50" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="C50" s="5"/>
-      <c r="D50" s="22" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="22" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="B52" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="22" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="32"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="22"/>
-    </row>
-    <row r="54" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="32"/>
-      <c r="B54" s="14"/>
-      <c r="C54"/>
-      <c r="D54" s="23"/>
-    </row>
-    <row r="55" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="32"/>
-      <c r="B55" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="C55" s="4"/>
-      <c r="D55" s="24"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="B56" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="D56" s="22" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B57" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C57" s="5"/>
-      <c r="D57" s="28" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="32" t="s">
-        <v>5</v>
-      </c>
-      <c r="B58" s="19" t="s">
+      <c r="B83" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="29" t="s">
+      <c r="C83" s="31" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A84" s="38"/>
+      <c r="B84" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="C84" s="31" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="32" t="s">
-        <v>6</v>
-      </c>
-      <c r="B59" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="22" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="32"/>
-      <c r="B60" s="14"/>
-      <c r="C60"/>
-      <c r="D60" s="23"/>
-    </row>
-    <row r="61" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="32"/>
-      <c r="B61" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D61" s="24"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B62" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C62" s="5"/>
-      <c r="D62" s="22" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="B63" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="22" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B64" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="22" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="B65" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="22" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B66" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C66" s="5"/>
-      <c r="D66" s="22" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="B67" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C67" s="5"/>
-      <c r="D67" s="22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B68" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="22" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B69" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="22" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A70" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B70" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="22" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="B71" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="22" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="B72" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="B73" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="29"/>
-    </row>
-    <row r="74" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A74" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="B74" s="14" t="s">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="38"/>
+      <c r="B85" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="28" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B75" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="22" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A76" s="31" t="s">
-        <v>116</v>
-      </c>
-      <c r="B76" s="14"/>
-      <c r="C76"/>
-      <c r="D76" s="23"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="B77" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C77" s="5"/>
-      <c r="D77" s="22" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A78" s="33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B78" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C78" s="5"/>
-      <c r="D78" s="28" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="32" t="s">
-        <v>5</v>
-      </c>
-      <c r="B79" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="C79" s="2"/>
-      <c r="D79" s="25"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="32" t="s">
-        <v>6</v>
-      </c>
-      <c r="B80" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C80" s="5"/>
-      <c r="D80" s="22" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A81" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="B81" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="C81" s="12"/>
-      <c r="D81" s="25" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="34" t="s">
+      <c r="C85" s="31" t="s">
         <v>200</v>
-      </c>
-      <c r="B82" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="C82" s="12"/>
-      <c r="D82" s="38"/>
-    </row>
-    <row r="83" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A83" s="42" t="s">
-        <v>201</v>
-      </c>
-      <c r="B83" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="C83" s="12"/>
-      <c r="D83" s="39" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A84" s="43"/>
-      <c r="B84" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="C84" s="12"/>
-      <c r="D84" s="39" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="43"/>
-      <c r="B85" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="C85" s="12"/>
-      <c r="D85" s="39" t="s">
-        <v>204</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A83:A85"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A83:A85"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B58" r:id="rId1" xr:uid="{4F261D28-2E5B-49F5-B0B7-CEFB3CF96721}"/>
-    <hyperlink ref="D58" r:id="rId2" xr:uid="{C079BE76-10DE-4C92-BE58-BD019A35A23A}"/>
-    <hyperlink ref="D81" r:id="rId3" display="https://www.samsung.com/n_africa/offer/" xr:uid="{4A920327-4AC0-4FC8-B4F5-F0B4E6A631F5}"/>
+    <hyperlink ref="C58" r:id="rId2" xr:uid="{C079BE76-10DE-4C92-BE58-BD019A35A23A}"/>
+    <hyperlink ref="C81" r:id="rId3" display="https://www.samsung.com/n_africa/offer/" xr:uid="{4A920327-4AC0-4FC8-B4F5-F0B4E6A631F5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
@@ -2248,13 +2156,13 @@
           <x14:formula1>
             <xm:f>Lists!$A$1:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>C4:D4</xm:sqref>
+          <xm:sqref>C4</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Lists!$B$2:$B$30</xm:f>
           </x14:formula1>
-          <xm:sqref>C5:D5</xm:sqref>
+          <xm:sqref>C5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2272,27 +2180,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
-        <v>64</v>
+      <c r="A1" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2314,188 +2222,188 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2507,6 +2415,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009E46DBE1B5DF38488B5DFC49E964C52B" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3559fc529dde5fb92138384961dffe22">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f461ead0-e9bd-4f0b-97d1-cf254b08f18b" xmlns:ns3="7df2ab9b-c382-483a-b5a6-0c5a88654256" xmlns:ns4="10221d51-6403-4ce2-acce-3db49615c262" xmlns:ns5="1fcb5b47-352b-4295-9c23-3c629ac97dad" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5935b0975cf95dc75073bcffc58f2424" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="f461ead0-e9bd-4f0b-97d1-cf254b08f18b"/>
@@ -2775,7 +2692,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <a8b37c27258c422e99a84a06d6491f40 xmlns="7df2ab9b-c382-483a-b5a6-0c5a88654256">
@@ -2806,16 +2723,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F3FB1A-7C57-4773-BE64-1F0955FDB0F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A8D01BA-0B69-493E-98A2-489910A9B93A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2836,7 +2752,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59E59CD1-F8B2-4B5A-91A2-8D54988138D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2846,12 +2762,4 @@
     <ds:schemaRef ds:uri="10221d51-6403-4ce2-acce-3db49615c262"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30F3FB1A-7C57-4773-BE64-1F0955FDB0F1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>